<commit_message>
Preference Logic Bug Fixed
</commit_message>
<xml_diff>
--- a/static/latest_schedule.xlsx
+++ b/static/latest_schedule.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Minal</t>
+          <t>Jonnah</t>
         </is>
       </c>
     </row>
@@ -475,7 +475,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Minjung</t>
+          <t>Mandy</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>yujin</t>
+          <t>Sam</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Sam</t>
+          <t>Minal</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sam</t>
+          <t>Minal</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Minal</t>
+          <t>yujin</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Jonnah</t>
+          <t>Minjung</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Seoyoon</t>
+          <t>Mandy</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fionna</t>
+          <t>Minjung</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Minjung</t>
+          <t>Fionna</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Mandy</t>
+          <t>Seoyoon</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fionna</t>
+          <t>Sam</t>
         </is>
       </c>
     </row>
@@ -713,7 +713,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Mandy</t>
+          <t>Sungwoo</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sungwoo</t>
+          <t>Fionna</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Name Clean for Parsing Excel
</commit_message>
<xml_diff>
--- a/static/latest_schedule.xlsx
+++ b/static/latest_schedule.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Jonnah</t>
+          <t>Jonnah✅</t>
         </is>
       </c>
     </row>
@@ -475,7 +475,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mandy</t>
+          <t>Mandy✅</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Jonnah</t>
+          <t>Jonnah✅</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sam</t>
+          <t>Sam✅</t>
         </is>
       </c>
     </row>
@@ -543,7 +543,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Sungwoo</t>
+          <t>Sungwoo✅</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Minal</t>
+          <t>Minal✅</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>yujin</t>
+          <t>yujin✅</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Mandy</t>
+          <t>Mandy✅</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Minal</t>
+          <t>Fionna✅</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Fionna</t>
+          <t>Minal✅</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>yujin</t>
+          <t>Seoyoon</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Seoyoon</t>
+          <t>yujin✅</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Sam</t>
+          <t>Sam✅</t>
         </is>
       </c>
     </row>
@@ -713,7 +713,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Sungwoo</t>
+          <t>Sungwoo✅</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Fionna</t>
+          <t>Fionna✅</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Final Working Version with Name Clean
</commit_message>
<xml_diff>
--- a/static/latest_schedule.xlsx
+++ b/static/latest_schedule.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Jonnah✅</t>
+          <t>Jonnah</t>
         </is>
       </c>
     </row>
@@ -475,7 +475,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mandy✅</t>
+          <t>Mandy</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Jonnah✅</t>
+          <t>Jonnah</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sam✅</t>
+          <t>Sam</t>
         </is>
       </c>
     </row>
@@ -543,7 +543,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Sungwoo✅</t>
+          <t>Sungwoo</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Minal✅</t>
+          <t>Minal</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>yujin✅</t>
+          <t>yujin</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Mandy✅</t>
+          <t>Mandy</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fionna✅</t>
+          <t>Minal</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Minal✅</t>
+          <t>Fionna</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>yujin✅</t>
+          <t>yujin</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Sam✅</t>
+          <t>Sam</t>
         </is>
       </c>
     </row>
@@ -713,7 +713,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Sungwoo✅</t>
+          <t>Sungwoo</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Fionna✅</t>
+          <t>Fionna</t>
         </is>
       </c>
     </row>

</xml_diff>